<commit_message>
Aplicar rango acordado 890–970 und (igual Chaqueta Lite) en LITE PANT
Mantiene curva de tallas, colores y ajustes de tienda del pant;
demanda teórica calculada queda como referencia en resumen.

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/LITE_PANT_RANGO_PRODUCCION.xlsx
+++ b/LITE_PANT_RANGO_PRODUCCION.xlsx
@@ -192,7 +192,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -271,9 +271,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -889,7 +886,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>── RANGO DE PRODUCCIÓN (CALCULADO) ──</t>
+          <t>── RANGO DE PRODUCCIÓN (ACORDADO — IGUAL CHAQUETA LITE) ──</t>
         </is>
       </c>
     </row>
@@ -900,7 +897,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>109</v>
+        <v>890</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -915,7 +912,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>153</v>
+        <v>970</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -930,7 +927,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>44</v>
+        <v>80</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -941,12 +938,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Base del rango</t>
+          <t>Demanda teórica calculada (referencia)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2.5–3.5 meses + SS 15%</t>
+          <t>109 – 153 und</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -1298,10 +1295,10 @@
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>15</v>
+        <v>118</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>20</v>
+        <v>129</v>
       </c>
     </row>
     <row r="6">
@@ -1316,10 +1313,10 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>28</v>
+        <v>229</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>39</v>
+        <v>249</v>
       </c>
     </row>
     <row r="7">
@@ -1334,10 +1331,10 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>32</v>
+        <v>265</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>45</v>
+        <v>288</v>
       </c>
     </row>
     <row r="8">
@@ -1352,10 +1349,10 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>21</v>
+        <v>174</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>30</v>
+        <v>189</v>
       </c>
     </row>
     <row r="9">
@@ -1370,10 +1367,10 @@
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>13</v>
+        <v>104</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>19</v>
+        <v>115</v>
       </c>
     </row>
     <row r="10">
@@ -1383,10 +1380,10 @@
         </is>
       </c>
       <c r="C10" s="10" t="n">
-        <v>109</v>
+        <v>890</v>
       </c>
       <c r="D10" s="10" t="n">
-        <v>153</v>
+        <v>970</v>
       </c>
     </row>
   </sheetData>
@@ -1430,14 +1427,14 @@
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
         <is>
-          <t>Rango producción: 109 – 153 und</t>
+          <t>Rango producción: 890 – 970 und</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
         <is>
-          <t>MÍNIMO — 109 und (compromiso)</t>
+          <t>MÍNIMO — 890 und (compromiso)</t>
         </is>
       </c>
     </row>
@@ -1485,22 +1482,22 @@
         </is>
       </c>
       <c r="B7" s="17" t="n">
-        <v>6</v>
+        <v>47</v>
       </c>
       <c r="C7" s="17" t="n">
-        <v>11</v>
+        <v>91</v>
       </c>
       <c r="D7" s="17" t="n">
-        <v>13</v>
+        <v>106</v>
       </c>
       <c r="E7" s="17" t="n">
-        <v>9</v>
+        <v>69</v>
       </c>
       <c r="F7" s="17" t="n">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="G7" s="17" t="n">
-        <v>44</v>
+        <v>356</v>
       </c>
     </row>
     <row r="8">
@@ -1510,22 +1507,22 @@
         </is>
       </c>
       <c r="B8" s="17" t="n">
-        <v>4</v>
+        <v>36</v>
       </c>
       <c r="C8" s="17" t="n">
-        <v>8</v>
+        <v>69</v>
       </c>
       <c r="D8" s="17" t="n">
-        <v>10</v>
+        <v>79</v>
       </c>
       <c r="E8" s="17" t="n">
-        <v>6</v>
+        <v>52</v>
       </c>
       <c r="F8" s="17" t="n">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="G8" s="17" t="n">
-        <v>33</v>
+        <v>267</v>
       </c>
     </row>
     <row r="9">
@@ -1535,22 +1532,22 @@
         </is>
       </c>
       <c r="B9" s="17" t="n">
-        <v>4</v>
+        <v>36</v>
       </c>
       <c r="C9" s="17" t="n">
-        <v>8</v>
+        <v>69</v>
       </c>
       <c r="D9" s="17" t="n">
-        <v>10</v>
+        <v>79</v>
       </c>
       <c r="E9" s="17" t="n">
-        <v>6</v>
+        <v>52</v>
       </c>
       <c r="F9" s="17" t="n">
-        <v>4</v>
+        <v>31</v>
       </c>
       <c r="G9" s="17" t="n">
-        <v>32</v>
+        <v>267</v>
       </c>
     </row>
     <row r="10">
@@ -1560,28 +1557,28 @@
         </is>
       </c>
       <c r="B10" s="19" t="n">
-        <v>14</v>
+        <v>119</v>
       </c>
       <c r="C10" s="19" t="n">
-        <v>27</v>
+        <v>229</v>
       </c>
       <c r="D10" s="19" t="n">
-        <v>33</v>
+        <v>264</v>
       </c>
       <c r="E10" s="19" t="n">
-        <v>21</v>
+        <v>173</v>
       </c>
       <c r="F10" s="19" t="n">
-        <v>14</v>
+        <v>105</v>
       </c>
       <c r="G10" s="19" t="n">
-        <v>109</v>
+        <v>890</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
         <is>
-          <t>MÁXIMO — 153 und (techo)</t>
+          <t>MÁXIMO — 970 und (techo)</t>
         </is>
       </c>
     </row>
@@ -1629,22 +1626,22 @@
         </is>
       </c>
       <c r="B14" s="17" t="n">
-        <v>8</v>
+        <v>52</v>
       </c>
       <c r="C14" s="17" t="n">
-        <v>16</v>
+        <v>100</v>
       </c>
       <c r="D14" s="17" t="n">
-        <v>18</v>
+        <v>115</v>
       </c>
       <c r="E14" s="17" t="n">
-        <v>12</v>
+        <v>76</v>
       </c>
       <c r="F14" s="17" t="n">
-        <v>7</v>
+        <v>45</v>
       </c>
       <c r="G14" s="17" t="n">
-        <v>61</v>
+        <v>388</v>
       </c>
     </row>
     <row r="15">
@@ -1654,22 +1651,22 @@
         </is>
       </c>
       <c r="B15" s="17" t="n">
-        <v>6</v>
+        <v>39</v>
       </c>
       <c r="C15" s="17" t="n">
-        <v>12</v>
+        <v>75</v>
       </c>
       <c r="D15" s="17" t="n">
-        <v>14</v>
+        <v>86</v>
       </c>
       <c r="E15" s="17" t="n">
-        <v>9</v>
+        <v>57</v>
       </c>
       <c r="F15" s="17" t="n">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="G15" s="17" t="n">
-        <v>46</v>
+        <v>291</v>
       </c>
     </row>
     <row r="16">
@@ -1679,22 +1676,22 @@
         </is>
       </c>
       <c r="B16" s="17" t="n">
-        <v>6</v>
+        <v>39</v>
       </c>
       <c r="C16" s="17" t="n">
-        <v>12</v>
+        <v>75</v>
       </c>
       <c r="D16" s="17" t="n">
-        <v>14</v>
+        <v>86</v>
       </c>
       <c r="E16" s="17" t="n">
-        <v>9</v>
+        <v>57</v>
       </c>
       <c r="F16" s="17" t="n">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="G16" s="17" t="n">
-        <v>46</v>
+        <v>291</v>
       </c>
     </row>
     <row r="17">
@@ -1704,22 +1701,22 @@
         </is>
       </c>
       <c r="B17" s="19" t="n">
-        <v>20</v>
+        <v>130</v>
       </c>
       <c r="C17" s="19" t="n">
-        <v>40</v>
+        <v>250</v>
       </c>
       <c r="D17" s="19" t="n">
-        <v>46</v>
+        <v>287</v>
       </c>
       <c r="E17" s="19" t="n">
-        <v>30</v>
+        <v>190</v>
       </c>
       <c r="F17" s="19" t="n">
-        <v>17</v>
+        <v>113</v>
       </c>
       <c r="G17" s="19" t="n">
-        <v>153</v>
+        <v>970</v>
       </c>
     </row>
     <row r="19">
@@ -1763,10 +1760,10 @@
         </is>
       </c>
       <c r="B21" s="22" t="n">
-        <v>68.48999999999999</v>
+        <v>554.16</v>
       </c>
       <c r="C21" s="23" t="n">
-        <v>94.90000000000001</v>
+        <v>603.6799999999999</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1786,10 +1783,10 @@
         </is>
       </c>
       <c r="B22" s="22" t="n">
-        <v>82.19</v>
+        <v>664.99</v>
       </c>
       <c r="C22" s="23" t="n">
-        <v>113.88</v>
+        <v>724.42</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1798,7 +1795,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>13.133 kg al máx</t>
+          <t>83.54 kg al máx</t>
         </is>
       </c>
     </row>
@@ -1809,10 +1806,10 @@
         </is>
       </c>
       <c r="B23" s="22" t="n">
-        <v>61.82</v>
+        <v>498.43</v>
       </c>
       <c r="C23" s="23" t="n">
-        <v>85.86</v>
+        <v>543.34</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1821,7 +1818,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>9.894 kg al máx</t>
+          <t>62.664 kg al máx</t>
         </is>
       </c>
     </row>
@@ -1832,10 +1829,10 @@
         </is>
       </c>
       <c r="B24" s="22" t="n">
-        <v>59.83</v>
+        <v>498.43</v>
       </c>
       <c r="C24" s="23" t="n">
-        <v>85.86</v>
+        <v>543.34</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1844,7 +1841,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>9.894 kg al máx</t>
+          <t>62.664 kg al máx</t>
         </is>
       </c>
     </row>
@@ -1855,10 +1852,10 @@
         </is>
       </c>
       <c r="B25" s="22" t="n">
-        <v>203.84</v>
+        <v>1661.86</v>
       </c>
       <c r="C25" s="23" t="n">
-        <v>285.6</v>
+        <v>1811.09</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1867,7 +1864,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>32.921 kg al máx · SS 20%</t>
+          <t>208.868 kg al máx · SS 20%</t>
         </is>
       </c>
     </row>
@@ -1878,10 +1875,10 @@
         </is>
       </c>
       <c r="B26" s="22" t="n">
-        <v>78.17</v>
+        <v>638.45</v>
       </c>
       <c r="C26" s="23" t="n">
-        <v>109.84</v>
+        <v>695.9</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1901,10 +1898,10 @@
         </is>
       </c>
       <c r="B27" s="22" t="n">
-        <v>109</v>
+        <v>890</v>
       </c>
       <c r="C27" s="23" t="n">
-        <v>153</v>
+        <v>970</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -1968,7 +1965,7 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Rango global: 109 – 153 und</t>
+          <t>Rango global: 890 – 970 und</t>
         </is>
       </c>
     </row>
@@ -2070,34 +2067,34 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>6</v>
+        <v>47</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>8</v>
+        <v>52</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>11</v>
+        <v>91</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>16</v>
+        <v>100</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>13</v>
+        <v>106</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>18</v>
+        <v>115</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>9</v>
+        <v>69</v>
       </c>
       <c r="I8" s="8" t="n">
-        <v>12</v>
+        <v>76</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="K8" s="8" t="n">
-        <v>7</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9">
@@ -2107,10 +2104,10 @@
         </is>
       </c>
       <c r="B9" s="10" t="n">
-        <v>44</v>
+        <v>356</v>
       </c>
       <c r="C9" s="10" t="n">
-        <v>61</v>
+        <v>388</v>
       </c>
     </row>
     <row r="11">
@@ -2211,34 +2208,34 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>4</v>
+        <v>36</v>
       </c>
       <c r="C14" s="8" t="n">
-        <v>6</v>
+        <v>39</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>8</v>
+        <v>69</v>
       </c>
       <c r="E14" s="8" t="n">
-        <v>12</v>
+        <v>75</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>10</v>
+        <v>79</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>14</v>
+        <v>86</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>6</v>
+        <v>52</v>
       </c>
       <c r="I14" s="8" t="n">
-        <v>9</v>
+        <v>57</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="K14" s="8" t="n">
-        <v>5</v>
+        <v>34</v>
       </c>
     </row>
     <row r="15">
@@ -2248,10 +2245,10 @@
         </is>
       </c>
       <c r="B15" s="10" t="n">
-        <v>33</v>
+        <v>267</v>
       </c>
       <c r="C15" s="10" t="n">
-        <v>46</v>
+        <v>291</v>
       </c>
     </row>
     <row r="17">
@@ -2352,34 +2349,34 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>4</v>
+        <v>36</v>
       </c>
       <c r="C20" s="8" t="n">
-        <v>6</v>
+        <v>39</v>
       </c>
       <c r="D20" s="7" t="n">
-        <v>8</v>
+        <v>69</v>
       </c>
       <c r="E20" s="8" t="n">
-        <v>12</v>
+        <v>75</v>
       </c>
       <c r="F20" s="7" t="n">
-        <v>10</v>
+        <v>79</v>
       </c>
       <c r="G20" s="8" t="n">
-        <v>14</v>
+        <v>86</v>
       </c>
       <c r="H20" s="7" t="n">
-        <v>6</v>
+        <v>52</v>
       </c>
       <c r="I20" s="8" t="n">
-        <v>9</v>
+        <v>57</v>
       </c>
       <c r="J20" s="7" t="n">
-        <v>4</v>
+        <v>31</v>
       </c>
       <c r="K20" s="8" t="n">
-        <v>5</v>
+        <v>34</v>
       </c>
     </row>
     <row r="21">
@@ -2389,10 +2386,10 @@
         </is>
       </c>
       <c r="B21" s="10" t="n">
-        <v>32</v>
+        <v>267</v>
       </c>
       <c r="C21" s="10" t="n">
-        <v>46</v>
+        <v>291</v>
       </c>
     </row>
     <row r="23">
@@ -2402,10 +2399,10 @@
         </is>
       </c>
       <c r="B23" s="10" t="n">
-        <v>109</v>
+        <v>890</v>
       </c>
       <c r="C23" s="10" t="n">
-        <v>153</v>
+        <v>970</v>
       </c>
     </row>
     <row r="25">
@@ -2422,10 +2419,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>44</v>
+        <v>356</v>
       </c>
       <c r="C26" t="n">
-        <v>61</v>
+        <v>388</v>
       </c>
     </row>
     <row r="27">
@@ -2435,10 +2432,10 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>33</v>
+        <v>267</v>
       </c>
       <c r="C27" t="n">
-        <v>46</v>
+        <v>291</v>
       </c>
     </row>
     <row r="28">
@@ -2448,10 +2445,10 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>32</v>
+        <v>267</v>
       </c>
       <c r="C28" t="n">
-        <v>46</v>
+        <v>291</v>
       </c>
     </row>
   </sheetData>
@@ -2578,28 +2575,28 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>44</v>
+        <v>356</v>
       </c>
       <c r="D5" t="n">
-        <v>61</v>
+        <v>388</v>
       </c>
       <c r="E5" t="n">
-        <v>68.48999999999999</v>
+        <v>554.16</v>
       </c>
       <c r="F5" t="n">
-        <v>94.90000000000001</v>
+        <v>603.6799999999999</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>82.19</v>
+        <v>664.99</v>
       </c>
       <c r="H5" s="8" t="n">
-        <v>113.88</v>
+        <v>724.42</v>
       </c>
       <c r="I5" s="22" t="n">
-        <v>9.475</v>
+        <v>76.71599999999999</v>
       </c>
       <c r="J5" s="23" t="n">
-        <v>13.133</v>
+        <v>83.54000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -2614,28 +2611,28 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>33</v>
+        <v>267</v>
       </c>
       <c r="D6" t="n">
-        <v>46</v>
+        <v>291</v>
       </c>
       <c r="E6" t="n">
-        <v>51.52</v>
+        <v>415.36</v>
       </c>
       <c r="F6" t="n">
-        <v>71.55</v>
+        <v>452.78</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>61.82</v>
+        <v>498.43</v>
       </c>
       <c r="H6" s="8" t="n">
-        <v>85.86</v>
+        <v>543.34</v>
       </c>
       <c r="I6" s="22" t="n">
-        <v>7.15</v>
+        <v>57.481</v>
       </c>
       <c r="J6" s="23" t="n">
-        <v>9.894</v>
+        <v>62.664</v>
       </c>
     </row>
     <row r="7">
@@ -2650,28 +2647,28 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>32</v>
+        <v>267</v>
       </c>
       <c r="D7" t="n">
-        <v>46</v>
+        <v>291</v>
       </c>
       <c r="E7" t="n">
-        <v>49.86</v>
+        <v>415.36</v>
       </c>
       <c r="F7" t="n">
-        <v>71.55</v>
+        <v>452.78</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>59.83</v>
+        <v>498.43</v>
       </c>
       <c r="H7" s="8" t="n">
-        <v>85.86</v>
+        <v>543.34</v>
       </c>
       <c r="I7" s="22" t="n">
-        <v>6.902</v>
+        <v>57.481</v>
       </c>
       <c r="J7" s="23" t="n">
-        <v>9.894</v>
+        <v>62.664</v>
       </c>
     </row>
     <row r="8">
@@ -2681,28 +2678,28 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>109</v>
+        <v>890</v>
       </c>
       <c r="D8" t="n">
-        <v>153</v>
+        <v>970</v>
       </c>
       <c r="E8" t="n">
-        <v>169.87</v>
+        <v>1384.88</v>
       </c>
       <c r="F8" t="n">
-        <v>238</v>
+        <v>1509.24</v>
       </c>
       <c r="G8" s="10" t="n">
-        <v>203.84</v>
+        <v>1661.86</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>285.6</v>
+        <v>1811.09</v>
       </c>
       <c r="I8" s="10" t="n">
-        <v>23.527</v>
+        <v>191.678</v>
       </c>
       <c r="J8" s="10" t="n">
-        <v>32.921</v>
+        <v>208.868</v>
       </c>
     </row>
     <row r="10">
@@ -2771,31 +2768,31 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>8</v>
+        <v>52</v>
       </c>
       <c r="C12" t="n">
-        <v>16</v>
+        <v>100</v>
       </c>
       <c r="D12" t="n">
-        <v>18</v>
+        <v>115</v>
       </c>
       <c r="E12" t="n">
-        <v>12</v>
+        <v>76</v>
       </c>
       <c r="F12" t="n">
-        <v>7</v>
+        <v>45</v>
       </c>
       <c r="G12" t="n">
-        <v>61</v>
+        <v>388</v>
       </c>
       <c r="H12" t="n">
-        <v>94.90000000000001</v>
+        <v>603.6799999999999</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>113.88</v>
+        <v>724.42</v>
       </c>
       <c r="J12" t="n">
-        <v>13.133</v>
+        <v>83.54000000000001</v>
       </c>
     </row>
     <row r="13">
@@ -2805,31 +2802,31 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>6</v>
+        <v>39</v>
       </c>
       <c r="C13" t="n">
-        <v>12</v>
+        <v>75</v>
       </c>
       <c r="D13" t="n">
-        <v>14</v>
+        <v>86</v>
       </c>
       <c r="E13" t="n">
-        <v>9</v>
+        <v>57</v>
       </c>
       <c r="F13" t="n">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="G13" t="n">
-        <v>46</v>
+        <v>291</v>
       </c>
       <c r="H13" t="n">
-        <v>71.55</v>
+        <v>452.78</v>
       </c>
       <c r="I13" s="8" t="n">
-        <v>85.86</v>
+        <v>543.34</v>
       </c>
       <c r="J13" t="n">
-        <v>9.894</v>
+        <v>62.664</v>
       </c>
     </row>
     <row r="14">
@@ -2839,31 +2836,31 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>6</v>
+        <v>39</v>
       </c>
       <c r="C14" t="n">
-        <v>12</v>
+        <v>75</v>
       </c>
       <c r="D14" t="n">
-        <v>14</v>
+        <v>86</v>
       </c>
       <c r="E14" t="n">
-        <v>9</v>
+        <v>57</v>
       </c>
       <c r="F14" t="n">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="G14" t="n">
-        <v>46</v>
+        <v>291</v>
       </c>
       <c r="H14" t="n">
-        <v>71.55</v>
+        <v>452.78</v>
       </c>
       <c r="I14" s="8" t="n">
-        <v>85.86</v>
+        <v>543.34</v>
       </c>
       <c r="J14" t="n">
-        <v>9.894</v>
+        <v>62.664</v>
       </c>
     </row>
     <row r="16">
@@ -2963,10 +2960,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>78.17</v>
+        <v>638.45</v>
       </c>
       <c r="C22" t="n">
-        <v>109.84</v>
+        <v>695.9</v>
       </c>
     </row>
     <row r="23">
@@ -2976,10 +2973,10 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>109</v>
+        <v>890</v>
       </c>
       <c r="C23" t="n">
-        <v>153</v>
+        <v>970</v>
       </c>
     </row>
   </sheetData>
@@ -3117,34 +3114,34 @@
         </is>
       </c>
       <c r="B5" s="22" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="C5" s="23" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="D5" s="22" t="n">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="E5" s="23" t="n">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="F5" s="22" t="n">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="G5" s="23" t="n">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="H5" s="22" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="I5" s="23" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="J5" s="22" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="K5" s="23" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6">
@@ -3154,34 +3151,34 @@
         </is>
       </c>
       <c r="B6" s="22" t="n">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="C6" s="23" t="n">
-        <v>4</v>
+        <v>27</v>
       </c>
       <c r="D6" s="22" t="n">
-        <v>5</v>
+        <v>48</v>
       </c>
       <c r="E6" s="23" t="n">
-        <v>8</v>
+        <v>52</v>
       </c>
       <c r="F6" s="22" t="n">
-        <v>6</v>
+        <v>56</v>
       </c>
       <c r="G6" s="23" t="n">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="H6" s="22" t="n">
-        <v>4</v>
+        <v>36</v>
       </c>
       <c r="I6" s="23" t="n">
-        <v>6</v>
+        <v>40</v>
       </c>
       <c r="J6" s="22" t="n">
-        <v>3</v>
+        <v>22</v>
       </c>
       <c r="K6" s="23" t="n">
-        <v>5</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7">
@@ -3191,34 +3188,34 @@
         </is>
       </c>
       <c r="B7" s="22" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="C7" s="23" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="D7" s="22" t="n">
-        <v>4</v>
+        <v>31</v>
       </c>
       <c r="E7" s="23" t="n">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="F7" s="22" t="n">
-        <v>4</v>
+        <v>36</v>
       </c>
       <c r="G7" s="23" t="n">
-        <v>6</v>
+        <v>39</v>
       </c>
       <c r="H7" s="22" t="n">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="I7" s="23" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="J7" s="22" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="K7" s="23" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8">
@@ -3228,34 +3225,34 @@
         </is>
       </c>
       <c r="B8" s="22" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="C8" s="23" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="D8" s="22" t="n">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="E8" s="23" t="n">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="F8" s="22" t="n">
-        <v>3</v>
+        <v>27</v>
       </c>
       <c r="G8" s="23" t="n">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="H8" s="22" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="I8" s="23" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="J8" s="22" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="K8" s="23" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9">
@@ -3264,35 +3261,35 @@
           <t>GRAND PLAZ ★</t>
         </is>
       </c>
-      <c r="B9" s="31" t="n">
-        <v>0</v>
+      <c r="B9" s="22" t="n">
+        <v>3</v>
       </c>
       <c r="C9" s="23" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D9" s="22" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E9" s="23" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F9" s="22" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G9" s="23" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="H9" s="22" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I9" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="J9" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" s="31" t="n">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="J9" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="K9" s="23" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -3302,34 +3299,34 @@
         </is>
       </c>
       <c r="B10" s="22" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="C10" s="23" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="D10" s="22" t="n">
-        <v>3</v>
+        <v>27</v>
       </c>
       <c r="E10" s="23" t="n">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="F10" s="22" t="n">
-        <v>4</v>
+        <v>32</v>
       </c>
       <c r="G10" s="23" t="n">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="H10" s="22" t="n">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="I10" s="23" t="n">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="J10" s="22" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="K10" s="23" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11">
@@ -3339,34 +3336,34 @@
         </is>
       </c>
       <c r="B11" s="22" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C11" s="23" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D11" s="22" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="E11" s="23" t="n">
-        <v>3</v>
+        <v>22</v>
       </c>
       <c r="F11" s="22" t="n">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="G11" s="23" t="n">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="H11" s="22" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="I11" s="23" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="J11" s="22" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="K11" s="23" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12">
@@ -3376,34 +3373,34 @@
         </is>
       </c>
       <c r="B12" s="22" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C12" s="23" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="D12" s="22" t="n">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="E12" s="23" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="F12" s="22" t="n">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="G12" s="23" t="n">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="H12" s="22" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="I12" s="23" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="J12" s="22" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="K12" s="23" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13">
@@ -3413,34 +3410,34 @@
         </is>
       </c>
       <c r="B13" s="22" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="C13" s="23" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="D13" s="22" t="n">
-        <v>4</v>
+        <v>31</v>
       </c>
       <c r="E13" s="23" t="n">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="F13" s="22" t="n">
-        <v>4</v>
+        <v>35</v>
       </c>
       <c r="G13" s="23" t="n">
-        <v>6</v>
+        <v>39</v>
       </c>
       <c r="H13" s="22" t="n">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="I13" s="23" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="J13" s="22" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="K13" s="23" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14">
@@ -3450,34 +3447,34 @@
         </is>
       </c>
       <c r="B14" s="10" t="n">
-        <v>14</v>
+        <v>119</v>
       </c>
       <c r="C14" s="10" t="n">
-        <v>21</v>
+        <v>127</v>
       </c>
       <c r="D14" s="10" t="n">
-        <v>28</v>
+        <v>229</v>
       </c>
       <c r="E14" s="10" t="n">
-        <v>38</v>
+        <v>248</v>
       </c>
       <c r="F14" s="10" t="n">
-        <v>32</v>
+        <v>264</v>
       </c>
       <c r="G14" s="10" t="n">
-        <v>46</v>
+        <v>289</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>22</v>
+        <v>172</v>
       </c>
       <c r="I14" s="10" t="n">
-        <v>30</v>
+        <v>189</v>
       </c>
       <c r="J14" s="10" t="n">
-        <v>13</v>
+        <v>106</v>
       </c>
       <c r="K14" s="10" t="n">
-        <v>18</v>
+        <v>117</v>
       </c>
     </row>
     <row r="16">
@@ -3516,10 +3513,10 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>12</v>
+        <v>94</v>
       </c>
       <c r="C18" t="n">
-        <v>16</v>
+        <v>103</v>
       </c>
       <c r="D18" t="n">
         <v>4.7</v>
@@ -3532,10 +3529,10 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>21</v>
+        <v>187</v>
       </c>
       <c r="C19" t="n">
-        <v>33</v>
+        <v>203</v>
       </c>
       <c r="D19" t="n">
         <v>9.4</v>
@@ -3548,10 +3545,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>15</v>
+        <v>120</v>
       </c>
       <c r="C20" t="n">
-        <v>21</v>
+        <v>130</v>
       </c>
       <c r="D20" t="n">
         <v>6</v>
@@ -3564,10 +3561,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>11</v>
+        <v>92</v>
       </c>
       <c r="C21" t="n">
-        <v>16</v>
+        <v>101</v>
       </c>
       <c r="D21" t="n">
         <v>4.6</v>
@@ -3580,10 +3577,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="C22" t="n">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="D22" t="n">
         <v>1.1</v>
@@ -3596,10 +3593,10 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>13</v>
+        <v>107</v>
       </c>
       <c r="C23" t="n">
-        <v>18</v>
+        <v>116</v>
       </c>
       <c r="D23" t="n">
         <v>5.4</v>
@@ -3612,10 +3609,10 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>10</v>
+        <v>78</v>
       </c>
       <c r="C24" t="n">
-        <v>13</v>
+        <v>86</v>
       </c>
       <c r="D24" t="n">
         <v>3.9</v>
@@ -3628,10 +3625,10 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>9</v>
+        <v>72</v>
       </c>
       <c r="C25" t="n">
-        <v>12</v>
+        <v>78</v>
       </c>
       <c r="D25" t="n">
         <v>3.6</v>
@@ -3644,10 +3641,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>15</v>
+        <v>119</v>
       </c>
       <c r="C26" t="n">
-        <v>20</v>
+        <v>130</v>
       </c>
       <c r="D26" t="n">
         <v>6</v>
@@ -3680,7 +3677,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="32" t="inlineStr">
+      <c r="A1" s="31" t="inlineStr">
         <is>
           <t>INSUMOS — LITE PANT DAMA</t>
         </is>
@@ -3737,10 +3734,10 @@
         <v>67</v>
       </c>
       <c r="C6" t="n">
-        <v>15</v>
+        <v>118</v>
       </c>
       <c r="D6" t="n">
-        <v>20</v>
+        <v>129</v>
       </c>
     </row>
     <row r="7">
@@ -3753,10 +3750,10 @@
         <v>69</v>
       </c>
       <c r="C7" t="n">
-        <v>28</v>
+        <v>229</v>
       </c>
       <c r="D7" t="n">
-        <v>39</v>
+        <v>249</v>
       </c>
     </row>
     <row r="8">
@@ -3769,10 +3766,10 @@
         <v>72</v>
       </c>
       <c r="C8" t="n">
-        <v>32</v>
+        <v>265</v>
       </c>
       <c r="D8" t="n">
-        <v>45</v>
+        <v>288</v>
       </c>
     </row>
     <row r="9">
@@ -3785,10 +3782,10 @@
         <v>75</v>
       </c>
       <c r="C9" t="n">
-        <v>21</v>
+        <v>174</v>
       </c>
       <c r="D9" t="n">
-        <v>30</v>
+        <v>189</v>
       </c>
     </row>
     <row r="10">
@@ -3801,10 +3798,10 @@
         <v>77</v>
       </c>
       <c r="C10" t="n">
-        <v>13</v>
+        <v>104</v>
       </c>
       <c r="D10" t="n">
-        <v>19</v>
+        <v>115</v>
       </c>
     </row>
     <row r="12">
@@ -3815,10 +3812,10 @@
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="n">
-        <v>78.17</v>
+        <v>638.45</v>
       </c>
       <c r="D12" t="n">
-        <v>109.84</v>
+        <v>695.9</v>
       </c>
     </row>
     <row r="14">
@@ -3857,7 +3854,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>109</v>
+        <v>890</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -3865,7 +3862,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>153</v>
+        <v>970</v>
       </c>
     </row>
     <row r="18">
@@ -3919,7 +3916,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>109 – 153 und</t>
+          <t>890 – 970 und</t>
         </is>
       </c>
     </row>
@@ -3941,7 +3938,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="33" t="inlineStr">
+      <c r="A1" s="32" t="inlineStr">
         <is>
           <t>METODOLOGÍA — PROYECCIÓN LITE PANT</t>
         </is>
@@ -4081,21 +4078,21 @@
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>4. RANGO DE PRODUCCIÓN</t>
+          <t>4. RANGO DE PRODUCCIÓN (ACORDADO)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Mínimo: 109 und | Máximo: 153 und.</t>
+          <t xml:space="preserve">   Mínimo: 890 und | Máximo: 970 und (mismo rango Chaqueta Lite).</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Calculado: 2.5–3.5 meses cobertura + SS 15%.</t>
+          <t xml:space="preserve">   Demanda teórica calculada: 109 – 153 und (referencia).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajustar curva tallas: +2 pp XS desde M en LITE PANT
Transferencia moderada M→XS sobre curva BASIC LINE PANT.
XS 13.3%→15.3% · M 29.7%→27.7% (≈+19 und XS al máx 970).

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/LITE_PANT_RANGO_PRODUCCION.xlsx
+++ b/LITE_PANT_RANGO_PRODUCCION.xlsx
@@ -639,7 +639,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C54"/>
+  <dimension ref="A1:C60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -1040,108 +1040,81 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>── AJUSTES DE TIENDA (DISTRIBUCIÓN) ──</t>
+          <t>── AJUSTE CURVA TALLAS ──</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Tolón histórico</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>und/mes</t>
-        </is>
-      </c>
+          <t>Curva histórica (BASIC LINE PANT)</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Dashboard Basic Line</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Tolón proyectado (85% Chacao)</t>
-        </is>
-      </c>
-      <c r="B40" t="n">
-        <v>3.9</v>
+          <t>Ajuste aplicado</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>+2 pp XS ← M</t>
+        </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>und/mes</t>
+          <t>refuerzo XS moderado</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Web histórica</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>und/mes</t>
-        </is>
-      </c>
+          <t>XS hist → ajustada</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>13.3% → 15.3%</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Web proyectada (60% Cerro Verde)</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>und/mes</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>La Vela histórica</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>und/mes</t>
-        </is>
-      </c>
+          <t>M hist → ajustada</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>29.7% → 27.7%</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>La Vela proyectada (avg Sambil + Cerro Verde)</t>
-        </is>
-      </c>
-      <c r="B44" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>und/mes</t>
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>── AJUSTES DE TIENDA (DISTRIBUCIÓN) ──</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Grand Plaz histórica</t>
+          <t>Tolón histórico</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1152,11 +1125,11 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Grand Plaz proyectada (+68% hist.)</t>
+          <t>Tolón proyectado (85% Chacao)</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>1.1</v>
+        <v>3.9</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1167,11 +1140,11 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Barquisimeto (avg Grieta+Chacao+Tolón proy.)</t>
+          <t>Web histórica</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>6</v>
+        <v>1.9</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1182,45 +1155,135 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Corporativo</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>EXCLUIDO</t>
+          <t>Web proyectada (60% Cerro Verde)</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>und/mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>La Vela histórica</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Notas</t>
+          <t>La Vela proyectada (avg Sambil + Cerro Verde)</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>• Referencia: BASIC LINE PANT DAMA del dashboard Basic Line.</t>
+          <t>Grand Plaz histórica</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>• Producto NUEVO manufacturado — sin stock inicial.</t>
+          <t>Grand Plaz proyectada (+68% hist.)</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>• Solo género DAMA, tallas XS a XL.</t>
+          <t>Barquisimeto (avg Grieta+Chacao+Tolón proy.)</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>6</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
+        <is>
+          <t>Corporativo</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>EXCLUIDO</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>• Referencia: BASIC LINE PANT DAMA del dashboard Basic Line.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>• Producto NUEVO manufacturado — sin stock inicial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>• Solo género DAMA, tallas XS a XL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
         <is>
           <t>• Compra tela VIORI incluye +20% stock de seguridad.</t>
         </is>
@@ -1291,14 +1354,14 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>13.3%</t>
+          <t>15.3%</t>
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>118</v>
+        <v>136</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>129</v>
+        <v>149</v>
       </c>
     </row>
     <row r="6">
@@ -1327,14 +1390,14 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>29.7%</t>
+          <t>27.7%</t>
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>265</v>
+        <v>247</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>288</v>
+        <v>269</v>
       </c>
     </row>
     <row r="8">
@@ -1370,7 +1433,7 @@
         <v>104</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="10">
@@ -1482,19 +1545,19 @@
         </is>
       </c>
       <c r="B7" s="17" t="n">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="C7" s="17" t="n">
         <v>91</v>
       </c>
       <c r="D7" s="17" t="n">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="E7" s="17" t="n">
         <v>69</v>
       </c>
       <c r="F7" s="17" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G7" s="17" t="n">
         <v>356</v>
@@ -1507,13 +1570,13 @@
         </is>
       </c>
       <c r="B8" s="17" t="n">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="C8" s="17" t="n">
         <v>69</v>
       </c>
       <c r="D8" s="17" t="n">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="E8" s="17" t="n">
         <v>52</v>
@@ -1532,13 +1595,13 @@
         </is>
       </c>
       <c r="B9" s="17" t="n">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="C9" s="17" t="n">
         <v>69</v>
       </c>
       <c r="D9" s="17" t="n">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="E9" s="17" t="n">
         <v>52</v>
@@ -1557,19 +1620,19 @@
         </is>
       </c>
       <c r="B10" s="19" t="n">
-        <v>119</v>
+        <v>137</v>
       </c>
       <c r="C10" s="19" t="n">
         <v>229</v>
       </c>
       <c r="D10" s="19" t="n">
-        <v>264</v>
+        <v>247</v>
       </c>
       <c r="E10" s="19" t="n">
         <v>173</v>
       </c>
       <c r="F10" s="19" t="n">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G10" s="19" t="n">
         <v>890</v>
@@ -1626,13 +1689,13 @@
         </is>
       </c>
       <c r="B14" s="17" t="n">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="C14" s="17" t="n">
         <v>100</v>
       </c>
       <c r="D14" s="17" t="n">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="E14" s="17" t="n">
         <v>76</v>
@@ -1651,19 +1714,19 @@
         </is>
       </c>
       <c r="B15" s="17" t="n">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="C15" s="17" t="n">
         <v>75</v>
       </c>
       <c r="D15" s="17" t="n">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="E15" s="17" t="n">
         <v>57</v>
       </c>
       <c r="F15" s="17" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G15" s="17" t="n">
         <v>291</v>
@@ -1676,19 +1739,19 @@
         </is>
       </c>
       <c r="B16" s="17" t="n">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="C16" s="17" t="n">
         <v>75</v>
       </c>
       <c r="D16" s="17" t="n">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="E16" s="17" t="n">
         <v>57</v>
       </c>
       <c r="F16" s="17" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G16" s="17" t="n">
         <v>291</v>
@@ -1701,19 +1764,19 @@
         </is>
       </c>
       <c r="B17" s="19" t="n">
-        <v>130</v>
+        <v>149</v>
       </c>
       <c r="C17" s="19" t="n">
         <v>250</v>
       </c>
       <c r="D17" s="19" t="n">
-        <v>287</v>
+        <v>270</v>
       </c>
       <c r="E17" s="19" t="n">
         <v>190</v>
       </c>
       <c r="F17" s="19" t="n">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="G17" s="19" t="n">
         <v>970</v>
@@ -1760,10 +1823,10 @@
         </is>
       </c>
       <c r="B21" s="22" t="n">
-        <v>554.16</v>
+        <v>553.04</v>
       </c>
       <c r="C21" s="23" t="n">
-        <v>603.6799999999999</v>
+        <v>602.77</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1783,10 +1846,10 @@
         </is>
       </c>
       <c r="B22" s="22" t="n">
-        <v>664.99</v>
+        <v>663.65</v>
       </c>
       <c r="C22" s="23" t="n">
-        <v>724.42</v>
+        <v>723.3200000000001</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1795,7 +1858,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>83.54 kg al máx</t>
+          <t>83.44 kg al máx</t>
         </is>
       </c>
     </row>
@@ -1806,10 +1869,10 @@
         </is>
       </c>
       <c r="B23" s="22" t="n">
-        <v>498.43</v>
+        <v>497.65</v>
       </c>
       <c r="C23" s="23" t="n">
-        <v>543.34</v>
+        <v>542.3</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1818,7 +1881,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>62.664 kg al máx</t>
+          <t>62.543 kg al máx</t>
         </is>
       </c>
     </row>
@@ -1829,10 +1892,10 @@
         </is>
       </c>
       <c r="B24" s="22" t="n">
-        <v>498.43</v>
+        <v>497.65</v>
       </c>
       <c r="C24" s="23" t="n">
-        <v>543.34</v>
+        <v>542.3</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1841,7 +1904,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>62.664 kg al máx</t>
+          <t>62.543 kg al máx</t>
         </is>
       </c>
     </row>
@@ -1852,10 +1915,10 @@
         </is>
       </c>
       <c r="B25" s="22" t="n">
-        <v>1661.86</v>
+        <v>1658.95</v>
       </c>
       <c r="C25" s="23" t="n">
-        <v>1811.09</v>
+        <v>1807.93</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1864,7 +1927,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>208.868 kg al máx · SS 20%</t>
+          <t>208.525 kg al máx · SS 20%</t>
         </is>
       </c>
     </row>
@@ -1875,10 +1938,10 @@
         </is>
       </c>
       <c r="B26" s="22" t="n">
-        <v>638.45</v>
+        <v>637.55</v>
       </c>
       <c r="C26" s="23" t="n">
-        <v>695.9</v>
+        <v>694.85</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -2067,10 +2130,10 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="D8" s="7" t="n">
         <v>91</v>
@@ -2079,10 +2142,10 @@
         <v>100</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="H8" s="7" t="n">
         <v>69</v>
@@ -2091,7 +2154,7 @@
         <v>76</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="K8" s="8" t="n">
         <v>45</v>
@@ -2208,10 +2271,10 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="C14" s="8" t="n">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="D14" s="7" t="n">
         <v>69</v>
@@ -2220,10 +2283,10 @@
         <v>75</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="H14" s="7" t="n">
         <v>52</v>
@@ -2235,7 +2298,7 @@
         <v>31</v>
       </c>
       <c r="K14" s="8" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="15">
@@ -2349,10 +2412,10 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="C20" s="8" t="n">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="D20" s="7" t="n">
         <v>69</v>
@@ -2361,10 +2424,10 @@
         <v>75</v>
       </c>
       <c r="F20" s="7" t="n">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="G20" s="8" t="n">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="H20" s="7" t="n">
         <v>52</v>
@@ -2376,7 +2439,7 @@
         <v>31</v>
       </c>
       <c r="K20" s="8" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="21">
@@ -2581,22 +2644,22 @@
         <v>388</v>
       </c>
       <c r="E5" t="n">
-        <v>554.16</v>
+        <v>553.04</v>
       </c>
       <c r="F5" t="n">
-        <v>603.6799999999999</v>
+        <v>602.77</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>664.99</v>
+        <v>663.65</v>
       </c>
       <c r="H5" s="8" t="n">
-        <v>724.42</v>
+        <v>723.3200000000001</v>
       </c>
       <c r="I5" s="22" t="n">
-        <v>76.71599999999999</v>
+        <v>76.566</v>
       </c>
       <c r="J5" s="23" t="n">
-        <v>83.54000000000001</v>
+        <v>83.44</v>
       </c>
     </row>
     <row r="6">
@@ -2617,22 +2680,22 @@
         <v>291</v>
       </c>
       <c r="E6" t="n">
-        <v>415.36</v>
+        <v>414.71</v>
       </c>
       <c r="F6" t="n">
-        <v>452.78</v>
+        <v>451.92</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>498.43</v>
+        <v>497.65</v>
       </c>
       <c r="H6" s="8" t="n">
-        <v>543.34</v>
+        <v>542.3</v>
       </c>
       <c r="I6" s="22" t="n">
-        <v>57.481</v>
+        <v>57.409</v>
       </c>
       <c r="J6" s="23" t="n">
-        <v>62.664</v>
+        <v>62.543</v>
       </c>
     </row>
     <row r="7">
@@ -2653,22 +2716,22 @@
         <v>291</v>
       </c>
       <c r="E7" t="n">
-        <v>415.36</v>
+        <v>414.71</v>
       </c>
       <c r="F7" t="n">
-        <v>452.78</v>
+        <v>451.92</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>498.43</v>
+        <v>497.65</v>
       </c>
       <c r="H7" s="8" t="n">
-        <v>543.34</v>
+        <v>542.3</v>
       </c>
       <c r="I7" s="22" t="n">
-        <v>57.481</v>
+        <v>57.409</v>
       </c>
       <c r="J7" s="23" t="n">
-        <v>62.664</v>
+        <v>62.543</v>
       </c>
     </row>
     <row r="8">
@@ -2684,22 +2747,22 @@
         <v>970</v>
       </c>
       <c r="E8" t="n">
-        <v>1384.88</v>
+        <v>1382.46</v>
       </c>
       <c r="F8" t="n">
-        <v>1509.24</v>
+        <v>1506.61</v>
       </c>
       <c r="G8" s="10" t="n">
-        <v>1661.86</v>
+        <v>1658.95</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>1811.09</v>
+        <v>1807.93</v>
       </c>
       <c r="I8" s="10" t="n">
-        <v>191.678</v>
+        <v>191.384</v>
       </c>
       <c r="J8" s="10" t="n">
-        <v>208.868</v>
+        <v>208.525</v>
       </c>
     </row>
     <row r="10">
@@ -2768,13 +2831,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="C12" t="n">
         <v>100</v>
       </c>
       <c r="D12" t="n">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="E12" t="n">
         <v>76</v>
@@ -2786,13 +2849,13 @@
         <v>388</v>
       </c>
       <c r="H12" t="n">
-        <v>603.6799999999999</v>
+        <v>602.77</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>724.42</v>
+        <v>723.3200000000001</v>
       </c>
       <c r="J12" t="n">
-        <v>83.54000000000001</v>
+        <v>83.44</v>
       </c>
     </row>
     <row r="13">
@@ -2802,31 +2865,31 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="C13" t="n">
         <v>75</v>
       </c>
       <c r="D13" t="n">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="E13" t="n">
         <v>57</v>
       </c>
       <c r="F13" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G13" t="n">
         <v>291</v>
       </c>
       <c r="H13" t="n">
-        <v>452.78</v>
+        <v>451.92</v>
       </c>
       <c r="I13" s="8" t="n">
-        <v>543.34</v>
+        <v>542.3</v>
       </c>
       <c r="J13" t="n">
-        <v>62.664</v>
+        <v>62.543</v>
       </c>
     </row>
     <row r="14">
@@ -2836,31 +2899,31 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="C14" t="n">
         <v>75</v>
       </c>
       <c r="D14" t="n">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="E14" t="n">
         <v>57</v>
       </c>
       <c r="F14" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G14" t="n">
         <v>291</v>
       </c>
       <c r="H14" t="n">
-        <v>452.78</v>
+        <v>451.92</v>
       </c>
       <c r="I14" s="8" t="n">
-        <v>543.34</v>
+        <v>542.3</v>
       </c>
       <c r="J14" t="n">
-        <v>62.664</v>
+        <v>62.543</v>
       </c>
     </row>
     <row r="16">
@@ -2960,10 +3023,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>638.45</v>
+        <v>637.55</v>
       </c>
       <c r="C22" t="n">
-        <v>695.9</v>
+        <v>694.85</v>
       </c>
     </row>
     <row r="23">
@@ -3114,10 +3177,10 @@
         </is>
       </c>
       <c r="B5" s="22" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C5" s="23" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D5" s="22" t="n">
         <v>24</v>
@@ -3126,10 +3189,10 @@
         <v>26</v>
       </c>
       <c r="F5" s="22" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G5" s="23" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="H5" s="22" t="n">
         <v>18</v>
@@ -3138,7 +3201,7 @@
         <v>20</v>
       </c>
       <c r="J5" s="22" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="K5" s="23" t="n">
         <v>12</v>
@@ -3151,10 +3214,10 @@
         </is>
       </c>
       <c r="B6" s="22" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C6" s="23" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="D6" s="22" t="n">
         <v>48</v>
@@ -3163,10 +3226,10 @@
         <v>52</v>
       </c>
       <c r="F6" s="22" t="n">
+        <v>52</v>
+      </c>
+      <c r="G6" s="23" t="n">
         <v>56</v>
-      </c>
-      <c r="G6" s="23" t="n">
-        <v>60</v>
       </c>
       <c r="H6" s="22" t="n">
         <v>36</v>
@@ -3188,10 +3251,10 @@
         </is>
       </c>
       <c r="B7" s="22" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C7" s="23" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D7" s="22" t="n">
         <v>31</v>
@@ -3200,10 +3263,10 @@
         <v>33</v>
       </c>
       <c r="F7" s="22" t="n">
+        <v>33</v>
+      </c>
+      <c r="G7" s="23" t="n">
         <v>36</v>
-      </c>
-      <c r="G7" s="23" t="n">
-        <v>39</v>
       </c>
       <c r="H7" s="22" t="n">
         <v>23</v>
@@ -3212,7 +3275,7 @@
         <v>25</v>
       </c>
       <c r="J7" s="22" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K7" s="23" t="n">
         <v>16</v>
@@ -3225,10 +3288,10 @@
         </is>
       </c>
       <c r="B8" s="22" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C8" s="23" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D8" s="22" t="n">
         <v>24</v>
@@ -3237,10 +3300,10 @@
         <v>26</v>
       </c>
       <c r="F8" s="22" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G8" s="23" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="H8" s="22" t="n">
         <v>18</v>
@@ -3249,7 +3312,7 @@
         <v>20</v>
       </c>
       <c r="J8" s="22" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="K8" s="23" t="n">
         <v>12</v>
@@ -3265,7 +3328,7 @@
         <v>3</v>
       </c>
       <c r="C9" s="23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D9" s="22" t="n">
         <v>5</v>
@@ -3277,7 +3340,7 @@
         <v>6</v>
       </c>
       <c r="G9" s="23" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H9" s="22" t="n">
         <v>4</v>
@@ -3299,10 +3362,10 @@
         </is>
       </c>
       <c r="B10" s="22" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C10" s="23" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D10" s="22" t="n">
         <v>27</v>
@@ -3311,10 +3374,10 @@
         <v>30</v>
       </c>
       <c r="F10" s="22" t="n">
+        <v>30</v>
+      </c>
+      <c r="G10" s="23" t="n">
         <v>32</v>
-      </c>
-      <c r="G10" s="23" t="n">
-        <v>34</v>
       </c>
       <c r="H10" s="22" t="n">
         <v>21</v>
@@ -3326,7 +3389,7 @@
         <v>13</v>
       </c>
       <c r="K10" s="23" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11">
@@ -3336,10 +3399,10 @@
         </is>
       </c>
       <c r="B11" s="22" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C11" s="23" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D11" s="22" t="n">
         <v>20</v>
@@ -3348,10 +3411,10 @@
         <v>22</v>
       </c>
       <c r="F11" s="22" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G11" s="23" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="H11" s="22" t="n">
         <v>15</v>
@@ -3360,7 +3423,7 @@
         <v>17</v>
       </c>
       <c r="J11" s="22" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="K11" s="23" t="n">
         <v>10</v>
@@ -3373,10 +3436,10 @@
         </is>
       </c>
       <c r="B12" s="22" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C12" s="23" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D12" s="22" t="n">
         <v>19</v>
@@ -3385,10 +3448,10 @@
         <v>20</v>
       </c>
       <c r="F12" s="22" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G12" s="23" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H12" s="22" t="n">
         <v>14</v>
@@ -3400,7 +3463,7 @@
         <v>8</v>
       </c>
       <c r="K12" s="23" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13">
@@ -3410,10 +3473,10 @@
         </is>
       </c>
       <c r="B13" s="22" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C13" s="23" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D13" s="22" t="n">
         <v>31</v>
@@ -3422,10 +3485,10 @@
         <v>33</v>
       </c>
       <c r="F13" s="22" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G13" s="23" t="n">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="H13" s="22" t="n">
         <v>23</v>
@@ -3447,10 +3510,10 @@
         </is>
       </c>
       <c r="B14" s="10" t="n">
-        <v>119</v>
+        <v>135</v>
       </c>
       <c r="C14" s="10" t="n">
-        <v>127</v>
+        <v>149</v>
       </c>
       <c r="D14" s="10" t="n">
         <v>229</v>
@@ -3459,10 +3522,10 @@
         <v>248</v>
       </c>
       <c r="F14" s="10" t="n">
-        <v>264</v>
+        <v>248</v>
       </c>
       <c r="G14" s="10" t="n">
-        <v>289</v>
+        <v>269</v>
       </c>
       <c r="H14" s="10" t="n">
         <v>172</v>
@@ -3474,7 +3537,7 @@
         <v>106</v>
       </c>
       <c r="K14" s="10" t="n">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="16">
@@ -3734,10 +3797,10 @@
         <v>67</v>
       </c>
       <c r="C6" t="n">
-        <v>118</v>
+        <v>136</v>
       </c>
       <c r="D6" t="n">
-        <v>129</v>
+        <v>149</v>
       </c>
     </row>
     <row r="7">
@@ -3766,10 +3829,10 @@
         <v>72</v>
       </c>
       <c r="C8" t="n">
-        <v>265</v>
+        <v>247</v>
       </c>
       <c r="D8" t="n">
-        <v>288</v>
+        <v>269</v>
       </c>
     </row>
     <row r="9">
@@ -3801,7 +3864,7 @@
         <v>104</v>
       </c>
       <c r="D10" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="12">
@@ -3812,10 +3875,10 @@
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="n">
-        <v>638.45</v>
+        <v>637.55</v>
       </c>
       <c r="D12" t="n">
-        <v>695.9</v>
+        <v>694.85</v>
       </c>
     </row>
     <row r="14">
@@ -3931,7 +3994,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A42"/>
+  <dimension ref="A1:A46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
@@ -4109,21 +4172,21 @@
     <row r="28">
       <c r="A28" s="12" t="inlineStr">
         <is>
-          <t>5. DISTRIBUCIÓN</t>
+          <t>5. AJUSTE CURVA TALLAS</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Por tienda: pesos mensuales proyectados (Tolón/Web/Barquisimeto ajustados).</t>
+          <t xml:space="preserve">   Curva histórica BASIC LINE PANT DAMA: XS 13.3% · M 29.7%.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Por talla: curva BASIC LINE PANT DAMA del dashboard.</t>
+          <t xml:space="preserve">   Ajuste fino: +2 pp a XS tomados de M → XS 15.3% · M 27.7%.</t>
         </is>
       </c>
     </row>
@@ -4133,71 +4196,95 @@
     <row r="32">
       <c r="A32" s="12" t="inlineStr">
         <is>
-          <t>6. COLORES Y COMPRA DE TELA</t>
+          <t>6. DISTRIBUCIÓN</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Colores producción: Negro 40% · Vinotinto 30% · Verde Militar 30%.</t>
+          <t xml:space="preserve">   Por tienda: pesos mensuales proyectados (Tolón/Web/Barquisimeto ajustados).</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Dentro de cada color se aplica la misma curva de tallas.</t>
+          <t xml:space="preserve">   Por talla: curva ajustada (ver sección 5).</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Consumo VIORI por pieza (ficha LITE PANT DAMA): XS 1.45m · S 1.48m · M 1.58m · L 1.63m · XL 1.66m.</t>
-        </is>
-      </c>
+      <c r="A35" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Stock de seguridad tela: +20% sobre consumo (compra = consumo × 1.2).</t>
+      <c r="A36" s="12" t="inlineStr">
+        <is>
+          <t>7. COLORES Y COMPRA DE TELA</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Ver hojas 'Producción Color × Talla' y 'Compra de Tela VIORI'.</t>
+          <t xml:space="preserve">   Colores producción: Negro 40% · Vinotinto 30% · Verde Militar 30%.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr"/>
+      <c r="A38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Dentro de cada color se aplica la misma curva de tallas.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="12" t="inlineStr">
-        <is>
-          <t>7. OTROS INSUMOS</t>
+      <c r="A39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Consumo VIORI por pieza (ficha LITE PANT DAMA): XS 1.45m · S 1.48m · M 1.58m · L 1.63m · XL 1.66m.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Elástica 4.5 cm: consumo por talla según ficha (67–77 cm/pieza).</t>
+          <t xml:space="preserve">   Stock de seguridad tela: +20% sobre consumo (compra = consumo × 1.2).</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t xml:space="preserve">   Ver hojas 'Producción Color × Talla' y 'Compra de Tela VIORI'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="12" t="inlineStr">
+        <is>
+          <t>8. OTROS INSUMOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Elástica 4.5 cm: consumo por talla según ficha (67–77 cm/pieza).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t xml:space="preserve">   Etiqueta agua/SENCAMER: 1 und/pieza · costado derecho.</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
+    <row r="46">
+      <c r="A46" t="inlineStr">
         <is>
           <t xml:space="preserve">   Hilos: Negro-N · Vinotinto · Verde Militar (según color de tela).</t>
         </is>

</xml_diff>

<commit_message>
Curva tallas LITE PANT: M 25%, S 22%, XS recibe resto de M+S
XS 13.3%→21.7% (+8.4 pp desde M y S). L/XL sin cambio.

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/LITE_PANT_RANGO_PRODUCCION.xlsx
+++ b/LITE_PANT_RANGO_PRODUCCION.xlsx
@@ -639,7 +639,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C60"/>
+  <dimension ref="A1:C61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -1060,76 +1060,86 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Ajuste aplicado</t>
+          <t>M objetivo</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>+2 pp XS ← M</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>refuerzo XS moderado</t>
+          <t>hist 29.7%</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>XS hist → ajustada</t>
+          <t>S objetivo</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>13.3% → 15.3%</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr"/>
+          <t>22%</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>hist 25.7%</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>M hist → ajustada</t>
+          <t>XS (recibe resto M+S)</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>29.7% → 27.7%</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
+          <t>21.7%</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>hist 13.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>L / XL</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Sin cambio</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>L 19.5% · XL 11.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
         <is>
           <t>── AJUSTES DE TIENDA (DISTRIBUCIÓN) ──</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Tolón histórico</t>
-        </is>
-      </c>
-      <c r="B45" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Tolón proyectado (85% Chacao)</t>
+          <t>Tolón histórico</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>3.9</v>
+        <v>0.7</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1140,11 +1150,11 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Web histórica</t>
+          <t>Tolón proyectado (85% Chacao)</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>1.9</v>
+        <v>3.9</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1155,11 +1165,11 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Web proyectada (60% Cerro Verde)</t>
+          <t>Web histórica</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>3.6</v>
+        <v>1.9</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1170,11 +1180,11 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>La Vela histórica</t>
+          <t>Web proyectada (60% Cerro Verde)</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>1.4</v>
+        <v>3.6</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1185,11 +1195,11 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>La Vela proyectada (avg Sambil + Cerro Verde)</t>
+          <t>La Vela histórica</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>5.4</v>
+        <v>1.4</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -1200,11 +1210,11 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Grand Plaz histórica</t>
+          <t>La Vela proyectada (avg Sambil + Cerro Verde)</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>0.6</v>
+        <v>5.4</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -1215,11 +1225,11 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Grand Plaz proyectada (+68% hist.)</t>
+          <t>Grand Plaz histórica</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>1.1</v>
+        <v>0.6</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -1230,11 +1240,11 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Barquisimeto (avg Grieta+Chacao+Tolón proy.)</t>
+          <t>Grand Plaz proyectada (+68% hist.)</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>6</v>
+        <v>1.1</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -1245,45 +1255,60 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
+          <t>Barquisimeto (avg Grieta+Chacao+Tolón proy.)</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>6</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>und/mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
           <t>Corporativo</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B55" t="inlineStr">
         <is>
           <t>EXCLUIDO</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>Notas</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>• Referencia: BASIC LINE PANT DAMA del dashboard Basic Line.</t>
+          <t>Notas</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>• Producto NUEVO manufacturado — sin stock inicial.</t>
+          <t>• Referencia: BASIC LINE PANT DAMA del dashboard Basic Line.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>• Solo género DAMA, tallas XS a XL.</t>
+          <t>• Producto NUEVO manufacturado — sin stock inicial.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
+        <is>
+          <t>• Solo género DAMA, tallas XS a XL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
         <is>
           <t>• Compra tela VIORI incluye +20% stock de seguridad.</t>
         </is>
@@ -1354,14 +1379,14 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>15.3%</t>
+          <t>21.7%</t>
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>136</v>
+        <v>193</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>149</v>
+        <v>211</v>
       </c>
     </row>
     <row r="6">
@@ -1372,14 +1397,14 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>25.7%</t>
+          <t>22.0%</t>
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>229</v>
+        <v>196</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>249</v>
+        <v>213</v>
       </c>
     </row>
     <row r="7">
@@ -1390,14 +1415,14 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>27.7%</t>
+          <t>25.0%</t>
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>247</v>
+        <v>222</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>269</v>
+        <v>242</v>
       </c>
     </row>
     <row r="8">
@@ -1430,10 +1455,10 @@
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="10">
@@ -1545,19 +1570,19 @@
         </is>
       </c>
       <c r="B7" s="17" t="n">
-        <v>55</v>
+        <v>77</v>
       </c>
       <c r="C7" s="17" t="n">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="D7" s="17" t="n">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="E7" s="17" t="n">
         <v>69</v>
       </c>
       <c r="F7" s="17" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G7" s="17" t="n">
         <v>356</v>
@@ -1570,13 +1595,13 @@
         </is>
       </c>
       <c r="B8" s="17" t="n">
-        <v>41</v>
+        <v>58</v>
       </c>
       <c r="C8" s="17" t="n">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="D8" s="17" t="n">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="E8" s="17" t="n">
         <v>52</v>
@@ -1595,13 +1620,13 @@
         </is>
       </c>
       <c r="B9" s="17" t="n">
-        <v>41</v>
+        <v>58</v>
       </c>
       <c r="C9" s="17" t="n">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="D9" s="17" t="n">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="E9" s="17" t="n">
         <v>52</v>
@@ -1620,19 +1645,19 @@
         </is>
       </c>
       <c r="B10" s="19" t="n">
-        <v>137</v>
+        <v>193</v>
       </c>
       <c r="C10" s="19" t="n">
-        <v>229</v>
+        <v>196</v>
       </c>
       <c r="D10" s="19" t="n">
-        <v>247</v>
+        <v>223</v>
       </c>
       <c r="E10" s="19" t="n">
         <v>173</v>
       </c>
       <c r="F10" s="19" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G10" s="19" t="n">
         <v>890</v>
@@ -1689,19 +1714,19 @@
         </is>
       </c>
       <c r="B14" s="17" t="n">
-        <v>59</v>
+        <v>84</v>
       </c>
       <c r="C14" s="17" t="n">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="D14" s="17" t="n">
-        <v>108</v>
+        <v>97</v>
       </c>
       <c r="E14" s="17" t="n">
         <v>76</v>
       </c>
       <c r="F14" s="17" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G14" s="17" t="n">
         <v>388</v>
@@ -1714,19 +1739,19 @@
         </is>
       </c>
       <c r="B15" s="17" t="n">
-        <v>45</v>
+        <v>63</v>
       </c>
       <c r="C15" s="17" t="n">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="D15" s="17" t="n">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="E15" s="17" t="n">
         <v>57</v>
       </c>
       <c r="F15" s="17" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G15" s="17" t="n">
         <v>291</v>
@@ -1739,19 +1764,19 @@
         </is>
       </c>
       <c r="B16" s="17" t="n">
-        <v>45</v>
+        <v>63</v>
       </c>
       <c r="C16" s="17" t="n">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="D16" s="17" t="n">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="E16" s="17" t="n">
         <v>57</v>
       </c>
       <c r="F16" s="17" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G16" s="17" t="n">
         <v>291</v>
@@ -1764,19 +1789,19 @@
         </is>
       </c>
       <c r="B17" s="19" t="n">
-        <v>149</v>
+        <v>210</v>
       </c>
       <c r="C17" s="19" t="n">
-        <v>250</v>
+        <v>213</v>
       </c>
       <c r="D17" s="19" t="n">
-        <v>270</v>
+        <v>243</v>
       </c>
       <c r="E17" s="19" t="n">
         <v>190</v>
       </c>
       <c r="F17" s="19" t="n">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="G17" s="19" t="n">
         <v>970</v>
@@ -1823,10 +1848,10 @@
         </is>
       </c>
       <c r="B21" s="22" t="n">
-        <v>553.04</v>
+        <v>551.5599999999999</v>
       </c>
       <c r="C21" s="23" t="n">
-        <v>602.77</v>
+        <v>601.1</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1846,10 +1871,10 @@
         </is>
       </c>
       <c r="B22" s="22" t="n">
-        <v>663.65</v>
+        <v>661.87</v>
       </c>
       <c r="C22" s="23" t="n">
-        <v>723.3200000000001</v>
+        <v>721.3200000000001</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1858,7 +1883,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>83.44 kg al máx</t>
+          <t>83.204 kg al máx</t>
         </is>
       </c>
     </row>
@@ -1869,10 +1894,10 @@
         </is>
       </c>
       <c r="B23" s="22" t="n">
-        <v>497.65</v>
+        <v>496.2</v>
       </c>
       <c r="C23" s="23" t="n">
-        <v>542.3</v>
+        <v>540.91</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1881,7 +1906,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>62.543 kg al máx</t>
+          <t>62.384 kg al máx</t>
         </is>
       </c>
     </row>
@@ -1892,10 +1917,10 @@
         </is>
       </c>
       <c r="B24" s="22" t="n">
-        <v>497.65</v>
+        <v>496.2</v>
       </c>
       <c r="C24" s="23" t="n">
-        <v>542.3</v>
+        <v>540.91</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1904,7 +1929,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>62.543 kg al máx</t>
+          <t>62.384 kg al máx</t>
         </is>
       </c>
     </row>
@@ -1915,10 +1940,10 @@
         </is>
       </c>
       <c r="B25" s="22" t="n">
-        <v>1658.95</v>
+        <v>1654.27</v>
       </c>
       <c r="C25" s="23" t="n">
-        <v>1807.93</v>
+        <v>1803.14</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1927,7 +1952,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>208.525 kg al máx · SS 20%</t>
+          <t>207.973 kg al máx · SS 20%</t>
         </is>
       </c>
     </row>
@@ -1938,10 +1963,10 @@
         </is>
       </c>
       <c r="B26" s="22" t="n">
-        <v>637.55</v>
+        <v>635.74</v>
       </c>
       <c r="C26" s="23" t="n">
-        <v>694.85</v>
+        <v>692.88</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -2130,22 +2155,22 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>55</v>
+        <v>77</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>59</v>
+        <v>84</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>108</v>
+        <v>97</v>
       </c>
       <c r="H8" s="7" t="n">
         <v>69</v>
@@ -2154,10 +2179,10 @@
         <v>76</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="K8" s="8" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9">
@@ -2271,22 +2296,22 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>41</v>
+        <v>58</v>
       </c>
       <c r="C14" s="8" t="n">
-        <v>45</v>
+        <v>63</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="E14" s="8" t="n">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="H14" s="7" t="n">
         <v>52</v>
@@ -2298,7 +2323,7 @@
         <v>31</v>
       </c>
       <c r="K14" s="8" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="15">
@@ -2412,22 +2437,22 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>41</v>
+        <v>58</v>
       </c>
       <c r="C20" s="8" t="n">
-        <v>45</v>
+        <v>63</v>
       </c>
       <c r="D20" s="7" t="n">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="E20" s="8" t="n">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="F20" s="7" t="n">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="G20" s="8" t="n">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="H20" s="7" t="n">
         <v>52</v>
@@ -2439,7 +2464,7 @@
         <v>31</v>
       </c>
       <c r="K20" s="8" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="21">
@@ -2644,22 +2669,22 @@
         <v>388</v>
       </c>
       <c r="E5" t="n">
-        <v>553.04</v>
+        <v>551.5599999999999</v>
       </c>
       <c r="F5" t="n">
-        <v>602.77</v>
+        <v>601.1</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>663.65</v>
+        <v>661.87</v>
       </c>
       <c r="H5" s="8" t="n">
-        <v>723.3200000000001</v>
+        <v>721.3200000000001</v>
       </c>
       <c r="I5" s="22" t="n">
-        <v>76.566</v>
+        <v>76.36199999999999</v>
       </c>
       <c r="J5" s="23" t="n">
-        <v>83.44</v>
+        <v>83.20399999999999</v>
       </c>
     </row>
     <row r="6">
@@ -2680,22 +2705,22 @@
         <v>291</v>
       </c>
       <c r="E6" t="n">
-        <v>414.71</v>
+        <v>413.5</v>
       </c>
       <c r="F6" t="n">
-        <v>451.92</v>
+        <v>450.76</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>497.65</v>
+        <v>496.2</v>
       </c>
       <c r="H6" s="8" t="n">
-        <v>542.3</v>
+        <v>540.91</v>
       </c>
       <c r="I6" s="22" t="n">
-        <v>57.409</v>
+        <v>57.224</v>
       </c>
       <c r="J6" s="23" t="n">
-        <v>62.543</v>
+        <v>62.384</v>
       </c>
     </row>
     <row r="7">
@@ -2716,22 +2741,22 @@
         <v>291</v>
       </c>
       <c r="E7" t="n">
-        <v>414.71</v>
+        <v>413.5</v>
       </c>
       <c r="F7" t="n">
-        <v>451.92</v>
+        <v>450.76</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>497.65</v>
+        <v>496.2</v>
       </c>
       <c r="H7" s="8" t="n">
-        <v>542.3</v>
+        <v>540.91</v>
       </c>
       <c r="I7" s="22" t="n">
-        <v>57.409</v>
+        <v>57.224</v>
       </c>
       <c r="J7" s="23" t="n">
-        <v>62.543</v>
+        <v>62.384</v>
       </c>
     </row>
     <row r="8">
@@ -2747,22 +2772,22 @@
         <v>970</v>
       </c>
       <c r="E8" t="n">
-        <v>1382.46</v>
+        <v>1378.56</v>
       </c>
       <c r="F8" t="n">
-        <v>1506.61</v>
+        <v>1502.62</v>
       </c>
       <c r="G8" s="10" t="n">
-        <v>1658.95</v>
+        <v>1654.27</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>1807.93</v>
+        <v>1803.14</v>
       </c>
       <c r="I8" s="10" t="n">
-        <v>191.384</v>
+        <v>190.811</v>
       </c>
       <c r="J8" s="10" t="n">
-        <v>208.525</v>
+        <v>207.973</v>
       </c>
     </row>
     <row r="10">
@@ -2831,31 +2856,31 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>59</v>
+        <v>84</v>
       </c>
       <c r="C12" t="n">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="D12" t="n">
-        <v>108</v>
+        <v>97</v>
       </c>
       <c r="E12" t="n">
         <v>76</v>
       </c>
       <c r="F12" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G12" t="n">
         <v>388</v>
       </c>
       <c r="H12" t="n">
-        <v>602.77</v>
+        <v>601.1</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>723.3200000000001</v>
+        <v>721.3200000000001</v>
       </c>
       <c r="J12" t="n">
-        <v>83.44</v>
+        <v>83.20399999999999</v>
       </c>
     </row>
     <row r="13">
@@ -2865,31 +2890,31 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>45</v>
+        <v>63</v>
       </c>
       <c r="C13" t="n">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="D13" t="n">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="E13" t="n">
         <v>57</v>
       </c>
       <c r="F13" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G13" t="n">
         <v>291</v>
       </c>
       <c r="H13" t="n">
-        <v>451.92</v>
+        <v>450.76</v>
       </c>
       <c r="I13" s="8" t="n">
-        <v>542.3</v>
+        <v>540.91</v>
       </c>
       <c r="J13" t="n">
-        <v>62.543</v>
+        <v>62.384</v>
       </c>
     </row>
     <row r="14">
@@ -2899,31 +2924,31 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>45</v>
+        <v>63</v>
       </c>
       <c r="C14" t="n">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="D14" t="n">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="E14" t="n">
         <v>57</v>
       </c>
       <c r="F14" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G14" t="n">
         <v>291</v>
       </c>
       <c r="H14" t="n">
-        <v>451.92</v>
+        <v>450.76</v>
       </c>
       <c r="I14" s="8" t="n">
-        <v>542.3</v>
+        <v>540.91</v>
       </c>
       <c r="J14" t="n">
-        <v>62.543</v>
+        <v>62.384</v>
       </c>
     </row>
     <row r="16">
@@ -3023,10 +3048,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>637.55</v>
+        <v>635.74</v>
       </c>
       <c r="C22" t="n">
-        <v>694.85</v>
+        <v>692.88</v>
       </c>
     </row>
     <row r="23">
@@ -3177,22 +3202,22 @@
         </is>
       </c>
       <c r="B5" s="22" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C5" s="23" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D5" s="22" t="n">
+        <v>21</v>
+      </c>
+      <c r="E5" s="23" t="n">
+        <v>23</v>
+      </c>
+      <c r="F5" s="22" t="n">
         <v>24</v>
       </c>
-      <c r="E5" s="23" t="n">
+      <c r="G5" s="23" t="n">
         <v>26</v>
-      </c>
-      <c r="F5" s="22" t="n">
-        <v>26</v>
-      </c>
-      <c r="G5" s="23" t="n">
-        <v>29</v>
       </c>
       <c r="H5" s="22" t="n">
         <v>18</v>
@@ -3201,7 +3226,7 @@
         <v>20</v>
       </c>
       <c r="J5" s="22" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="K5" s="23" t="n">
         <v>12</v>
@@ -3214,22 +3239,22 @@
         </is>
       </c>
       <c r="B6" s="22" t="n">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="C6" s="23" t="n">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="D6" s="22" t="n">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="E6" s="23" t="n">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="F6" s="22" t="n">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="G6" s="23" t="n">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="H6" s="22" t="n">
         <v>36</v>
@@ -3241,7 +3266,7 @@
         <v>22</v>
       </c>
       <c r="K6" s="23" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7">
@@ -3251,22 +3276,22 @@
         </is>
       </c>
       <c r="B7" s="22" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="C7" s="23" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="D7" s="22" t="n">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="E7" s="23" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="F7" s="22" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="G7" s="23" t="n">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="H7" s="22" t="n">
         <v>23</v>
@@ -3288,22 +3313,22 @@
         </is>
       </c>
       <c r="B8" s="22" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C8" s="23" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="D8" s="22" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="E8" s="23" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="F8" s="22" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="G8" s="23" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="H8" s="22" t="n">
         <v>18</v>
@@ -3312,7 +3337,7 @@
         <v>20</v>
       </c>
       <c r="J8" s="22" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K8" s="23" t="n">
         <v>12</v>
@@ -3325,19 +3350,19 @@
         </is>
       </c>
       <c r="B9" s="22" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C9" s="23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D9" s="22" t="n">
         <v>5</v>
       </c>
       <c r="E9" s="23" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F9" s="22" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G9" s="23" t="n">
         <v>6</v>
@@ -3349,7 +3374,7 @@
         <v>4</v>
       </c>
       <c r="J9" s="22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K9" s="23" t="n">
         <v>3</v>
@@ -3362,22 +3387,22 @@
         </is>
       </c>
       <c r="B10" s="22" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="C10" s="23" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="D10" s="22" t="n">
+        <v>24</v>
+      </c>
+      <c r="E10" s="23" t="n">
+        <v>26</v>
+      </c>
+      <c r="F10" s="22" t="n">
         <v>27</v>
       </c>
-      <c r="E10" s="23" t="n">
-        <v>30</v>
-      </c>
-      <c r="F10" s="22" t="n">
-        <v>30</v>
-      </c>
       <c r="G10" s="23" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="H10" s="22" t="n">
         <v>21</v>
@@ -3386,7 +3411,7 @@
         <v>23</v>
       </c>
       <c r="J10" s="22" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K10" s="23" t="n">
         <v>13</v>
@@ -3399,22 +3424,22 @@
         </is>
       </c>
       <c r="B11" s="22" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C11" s="23" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="D11" s="22" t="n">
+        <v>17</v>
+      </c>
+      <c r="E11" s="23" t="n">
+        <v>19</v>
+      </c>
+      <c r="F11" s="22" t="n">
         <v>20</v>
       </c>
-      <c r="E11" s="23" t="n">
+      <c r="G11" s="23" t="n">
         <v>22</v>
-      </c>
-      <c r="F11" s="22" t="n">
-        <v>22</v>
-      </c>
-      <c r="G11" s="23" t="n">
-        <v>24</v>
       </c>
       <c r="H11" s="22" t="n">
         <v>15</v>
@@ -3426,7 +3451,7 @@
         <v>9</v>
       </c>
       <c r="K11" s="23" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12">
@@ -3436,22 +3461,22 @@
         </is>
       </c>
       <c r="B12" s="22" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C12" s="23" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="D12" s="22" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E12" s="23" t="n">
+        <v>17</v>
+      </c>
+      <c r="F12" s="22" t="n">
+        <v>18</v>
+      </c>
+      <c r="G12" s="23" t="n">
         <v>20</v>
-      </c>
-      <c r="F12" s="22" t="n">
-        <v>20</v>
-      </c>
-      <c r="G12" s="23" t="n">
-        <v>22</v>
       </c>
       <c r="H12" s="22" t="n">
         <v>14</v>
@@ -3473,22 +3498,22 @@
         </is>
       </c>
       <c r="B13" s="22" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="C13" s="23" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="D13" s="22" t="n">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="E13" s="23" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="F13" s="22" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="G13" s="23" t="n">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="H13" s="22" t="n">
         <v>23</v>
@@ -3510,22 +3535,22 @@
         </is>
       </c>
       <c r="B14" s="10" t="n">
-        <v>135</v>
+        <v>194</v>
       </c>
       <c r="C14" s="10" t="n">
-        <v>149</v>
+        <v>210</v>
       </c>
       <c r="D14" s="10" t="n">
-        <v>229</v>
+        <v>196</v>
       </c>
       <c r="E14" s="10" t="n">
-        <v>248</v>
+        <v>215</v>
       </c>
       <c r="F14" s="10" t="n">
-        <v>248</v>
+        <v>224</v>
       </c>
       <c r="G14" s="10" t="n">
-        <v>269</v>
+        <v>243</v>
       </c>
       <c r="H14" s="10" t="n">
         <v>172</v>
@@ -3534,10 +3559,10 @@
         <v>189</v>
       </c>
       <c r="J14" s="10" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="K14" s="10" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="16">
@@ -3797,10 +3822,10 @@
         <v>67</v>
       </c>
       <c r="C6" t="n">
-        <v>136</v>
+        <v>193</v>
       </c>
       <c r="D6" t="n">
-        <v>149</v>
+        <v>211</v>
       </c>
     </row>
     <row r="7">
@@ -3813,10 +3838,10 @@
         <v>69</v>
       </c>
       <c r="C7" t="n">
-        <v>229</v>
+        <v>196</v>
       </c>
       <c r="D7" t="n">
-        <v>249</v>
+        <v>213</v>
       </c>
     </row>
     <row r="8">
@@ -3829,10 +3854,10 @@
         <v>72</v>
       </c>
       <c r="C8" t="n">
-        <v>247</v>
+        <v>222</v>
       </c>
       <c r="D8" t="n">
-        <v>269</v>
+        <v>242</v>
       </c>
     </row>
     <row r="9">
@@ -3861,10 +3886,10 @@
         <v>77</v>
       </c>
       <c r="C10" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D10" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="12">
@@ -3875,10 +3900,10 @@
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="n">
-        <v>637.55</v>
+        <v>635.74</v>
       </c>
       <c r="D12" t="n">
-        <v>694.85</v>
+        <v>692.88</v>
       </c>
     </row>
     <row r="14">
@@ -3994,7 +4019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A46"/>
+  <dimension ref="A1:A47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
@@ -4179,112 +4204,119 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Curva histórica BASIC LINE PANT DAMA: XS 13.3% · M 29.7%.</t>
+          <t xml:space="preserve">   Histórica: XS 13.3% · S 25.7% · M 29.7%.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Ajuste fino: +2 pp a XS tomados de M → XS 15.3% · M 27.7%.</t>
+          <t xml:space="preserve">   Ajustada: M 25% · S 22% · XS 21.7% (recibe lo restado de M y S).</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr"/>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   L/XL sin cambio: 19.5% · 11.8%.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="12" t="inlineStr">
+      <c r="A32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="inlineStr">
         <is>
           <t>6. DISTRIBUCIÓN</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Por tienda: pesos mensuales proyectados (Tolón/Web/Barquisimeto ajustados).</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t xml:space="preserve">   Por tienda: pesos mensuales proyectados (Tolón/Web/Barquisimeto ajustados).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t xml:space="preserve">   Por talla: curva ajustada (ver sección 5).</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="inlineStr"/>
-    </row>
     <row r="36">
-      <c r="A36" s="12" t="inlineStr">
+      <c r="A36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="12" t="inlineStr">
         <is>
           <t>7. COLORES Y COMPRA DE TELA</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Colores producción: Negro 40% · Vinotinto 30% · Verde Militar 30%.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Dentro de cada color se aplica la misma curva de tallas.</t>
+          <t xml:space="preserve">   Colores producción: Negro 40% · Vinotinto 30% · Verde Militar 30%.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Consumo VIORI por pieza (ficha LITE PANT DAMA): XS 1.45m · S 1.48m · M 1.58m · L 1.63m · XL 1.66m.</t>
+          <t xml:space="preserve">   Dentro de cada color se aplica la misma curva de tallas.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Stock de seguridad tela: +20% sobre consumo (compra = consumo × 1.2).</t>
+          <t xml:space="preserve">   Consumo VIORI por pieza (ficha LITE PANT DAMA): XS 1.45m · S 1.48m · M 1.58m · L 1.63m · XL 1.66m.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t xml:space="preserve">   Stock de seguridad tela: +20% sobre consumo (compra = consumo × 1.2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t xml:space="preserve">   Ver hojas 'Producción Color × Talla' y 'Compra de Tela VIORI'.</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" t="inlineStr"/>
-    </row>
     <row r="43">
-      <c r="A43" s="12" t="inlineStr">
+      <c r="A43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="12" t="inlineStr">
         <is>
           <t>8. OTROS INSUMOS</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Elástica 4.5 cm: consumo por talla según ficha (67–77 cm/pieza).</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Etiqueta agua/SENCAMER: 1 und/pieza · costado derecho.</t>
+          <t xml:space="preserve">   Elástica 4.5 cm: consumo por talla según ficha (67–77 cm/pieza).</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Etiqueta agua/SENCAMER: 1 und/pieza · costado derecho.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
         <is>
           <t xml:space="preserve">   Hilos: Negro-N · Vinotinto · Verde Militar (según color de tela).</t>
         </is>

</xml_diff>